<commit_message>
Add one field in contract renewal
</commit_message>
<xml_diff>
--- a/Contract MasterData.xlsx
+++ b/Contract MasterData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MCT\Margi - Real Estate Dev\BRE-Property-Management-Margi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8D311F-BBA4-45DA-ABEF-093FDC9A2C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8528CB3C-8E4E-413D-9FF1-5ABE70147219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -139,7 +139,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -156,35 +156,44 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="8">
     <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -207,76 +216,6 @@
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -291,35 +230,35 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="Data" displayName="Data" ref="A1:X2" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="Data" displayName="Data" ref="A1:X2" totalsRowShown="0" headerRowDxfId="0" dataDxfId="7">
   <autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Report_Period" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Owner_s_Name" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Customer_Name" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Start_Date" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_End_Date" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Type" dataDxfId="20"/>
-    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Proposal_ID" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Tenor" dataDxfId="18"/>
-    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Contract_Status" dataDxfId="17"/>
-    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Amount" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Annual_Rent_Amount" dataDxfId="15"/>
-    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Security_Deposit_Amount" dataDxfId="14"/>
-    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Property_Name" dataDxfId="13"/>
-    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Name" dataDxfId="12"/>
-    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitID" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Number" dataDxfId="10"/>
-    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitArea_Sq_Feet" dataDxfId="9"/>
-    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Usage_Type" dataDxfId="8"/>
-    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspension_Date" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspended_Reason_list" dataDxfId="6"/>
-    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Start_Date" dataDxfId="5"/>
-    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_End_Date" dataDxfId="4"/>
-    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Period" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Report_Period" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID" dataCellStyle="Normal"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Owner_s_Name" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Customer_Name" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Start_Date" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_End_Date" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Type" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Proposal_ID" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Tenor" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Contract_Status" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Amount" dataCellStyle="Normal"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Annual_Rent_Amount" dataCellStyle="Normal"/>
+    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Security_Deposit_Amount" dataCellStyle="Normal"/>
+    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Property_Name" dataCellStyle="Normal"/>
+    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Name" dataCellStyle="Normal"/>
+    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitID" dataCellStyle="Normal"/>
+    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Number" dataCellStyle="Normal"/>
+    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitArea_Sq_Feet" dataCellStyle="Normal"/>
+    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Usage_Type" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspension_Date" dataDxfId="5"/>
+    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspended_Reason_list" dataDxfId="4"/>
+    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Start_Date" dataDxfId="3"/>
+    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_End_Date" dataDxfId="2"/>
+    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Period" dataDxfId="1"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -647,88 +586,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="6">
+      <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
         <v>24</v>
       </c>
       <c r="E2" t="s">
@@ -770,7 +708,7 @@
       <c r="Q2" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="3">
+      <c r="R2">
         <v>0</v>
       </c>
       <c r="S2" t="s">
@@ -788,7 +726,7 @@
       <c r="W2" t="s">
         <v>24</v>
       </c>
-      <c r="X2" s="5">
+      <c r="X2" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added a changes in contract master data and termination template
</commit_message>
<xml_diff>
--- a/Contract MasterData.xlsx
+++ b/Contract MasterData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\MCT\Margi - Real Estate Dev\BRE-Property-Management-Margi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8528CB3C-8E4E-413D-9FF1-5ABE70147219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F49385D-26FF-436F-B4F0-458F5900D531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +25,7 @@
     <definedName name="ReportMetadata.ObjectID" comment="Use this function to get the Object ID from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object ID",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportMetadata.ObjectName" comment="Use this function to get the Object Name from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Object Name",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportMetadata.ReportHelpLink" comment="Use this function to get the Report help link from the ReportMetadataValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Report help link",#REF!,#REF!,"none",)</definedName>
+    <definedName name="ReportRequest.CompanyDisplayName" comment="Use this function to get the Company display name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company display name",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.CompanyId" comment="Use this function to get the Company Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company Id",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.CompanyName" comment="Use this function to get the Company name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Company name",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.Date" comment="Use this function to get the Date from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Date",#REF!,#REF!,"none",)</definedName>
@@ -32,16 +33,32 @@
     <definedName name="ReportRequest.EnvironmentType" comment="Use this function to get the Environment type from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Environment type",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.FormatRegion" comment="Use this function to get the Format Region from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Format Region",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.Language" comment="Use this function to get the Language from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Language",#REF!,#REF!,"none",)</definedName>
+    <definedName name="ReportRequest.LayoutCaption" comment="Use this function to get the Layout caption from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout caption",#REF!,#REF!,"none",)</definedName>
+    <definedName name="ReportRequest.LayoutId" comment="Use this function to get the Layout id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout id",#REF!,#REF!,"none",)</definedName>
+    <definedName name="ReportRequest.LayoutName" comment="Use this function to get the Layout name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Layout name",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.TenantEntraId" comment="Use this function to get the Tenant Entra Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Entra Id",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.TenantId" comment="Use this function to get the Tenant Id from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("Tenant Id",#REF!,#REF!,"none",)</definedName>
     <definedName name="ReportRequest.UserName" comment="Use this function to get the User name from the ReportRequestValues table in the Aggregated Metadata worksheet">_xlfn.XLOOKUP("User name",#REF!,#REF!,"none",)</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
   <si>
     <t>Report_Period</t>
   </si>
@@ -113,6 +130,9 @@
   </si>
   <si>
     <t>Grace_Period</t>
+  </si>
+  <si>
+    <t>Termination_Date</t>
   </si>
   <si>
     <t/>
@@ -130,18 +150,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -158,18 +172,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="1">
     <dxf>
       <font>
         <b/>
@@ -191,30 +201,9 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
+          <bgColor rgb="FFC0C0C0"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -230,33 +219,34 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="Data" displayName="Data" ref="A1:X2" totalsRowShown="0" headerRowDxfId="0" dataDxfId="7">
-  <autoFilter ref="A1:X2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
-  <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Report_Period" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID" dataCellStyle="Normal"/>
-    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Owner_s_Name" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Customer_Name" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Start_Date" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_End_Date" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Type" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Proposal_ID" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Tenor" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Contract_Status" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Amount" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Annual_Rent_Amount" dataCellStyle="Normal"/>
-    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Security_Deposit_Amount" dataCellStyle="Normal"/>
-    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Property_Name" dataCellStyle="Normal"/>
-    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Name" dataCellStyle="Normal"/>
-    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitID" dataCellStyle="Normal"/>
-    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Number" dataCellStyle="Normal"/>
-    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitArea_Sq_Feet" dataCellStyle="Normal"/>
-    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Usage_Type" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspension_Date" dataDxfId="5"/>
-    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspended_Reason_list" dataDxfId="4"/>
-    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Start_Date" dataDxfId="3"/>
-    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_End_Date" dataDxfId="2"/>
-    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Period" dataDxfId="1"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}" name="Data" displayName="Data" ref="A1:Y2" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:Y2" xr:uid="{41D726F2-778D-4B1C-A5EA-875FED73D050}"/>
+  <tableColumns count="25">
+    <tableColumn id="1" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Report_Period"/>
+    <tableColumn id="2" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_ID"/>
+    <tableColumn id="3" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Owner_s_Name"/>
+    <tableColumn id="4" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Customer_Name"/>
+    <tableColumn id="5" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Start_Date"/>
+    <tableColumn id="6" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_End_Date"/>
+    <tableColumn id="7" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Type"/>
+    <tableColumn id="8" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Proposal_ID"/>
+    <tableColumn id="9" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Tenor"/>
+    <tableColumn id="10" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Tenant_Contract_Status"/>
+    <tableColumn id="11" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Contract_Amount"/>
+    <tableColumn id="12" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Annual_Rent_Amount"/>
+    <tableColumn id="13" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Security_Deposit_Amount"/>
+    <tableColumn id="14" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Property_Name"/>
+    <tableColumn id="15" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Name"/>
+    <tableColumn id="16" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitID"/>
+    <tableColumn id="17" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Number"/>
+    <tableColumn id="18" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="UnitArea_Sq_Feet"/>
+    <tableColumn id="19" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Unit_Usage_Type"/>
+    <tableColumn id="20" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspension_Date"/>
+    <tableColumn id="21" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Suspended_Reason_list"/>
+    <tableColumn id="22" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Start_Date"/>
+    <tableColumn id="23" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_End_Date"/>
+    <tableColumn id="24" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Grace_Period"/>
+    <tableColumn id="25" xr3:uid="{21867904-D69E-41E3-B5BE-D9B124B8D7E4}" name="Termination_Date"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -559,174 +549,187 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X2"/>
-  <sheetFormatPr defaultColWidth="25.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Y2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.109375" customWidth="1"/>
-    <col min="2" max="2" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" customWidth="1"/>
-    <col min="5" max="5" width="20.77734375" customWidth="1"/>
-    <col min="6" max="6" width="19.77734375" customWidth="1"/>
-    <col min="7" max="7" width="19.33203125" customWidth="1"/>
-    <col min="10" max="10" width="24.77734375" customWidth="1"/>
-    <col min="11" max="11" width="19.88671875" customWidth="1"/>
-    <col min="12" max="12" width="22.6640625" customWidth="1"/>
-    <col min="14" max="14" width="22.5546875" customWidth="1"/>
-    <col min="15" max="15" width="15.21875" customWidth="1"/>
-    <col min="16" max="16" width="10" customWidth="1"/>
-    <col min="17" max="17" width="15.6640625" customWidth="1"/>
-    <col min="18" max="18" width="19.88671875" customWidth="1"/>
-    <col min="19" max="19" width="18.33203125" customWidth="1"/>
-    <col min="20" max="20" width="19.109375" customWidth="1"/>
-    <col min="21" max="21" width="23.88671875" customWidth="1"/>
-    <col min="22" max="22" width="18.44140625" customWidth="1"/>
-    <col min="23" max="23" width="18.5546875" customWidth="1"/>
-    <col min="24" max="24" width="15.88671875" customWidth="1"/>
+    <col min="1" max="1" width="21.21875" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="7" max="7" width="23.88671875" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="17.21875" customWidth="1"/>
+    <col min="10" max="10" width="23.88671875" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" customWidth="1"/>
+    <col min="12" max="12" width="23.21875" customWidth="1"/>
+    <col min="13" max="13" width="26.44140625" customWidth="1"/>
+    <col min="14" max="14" width="17.21875" customWidth="1"/>
+    <col min="15" max="15" width="16.109375" customWidth="1"/>
+    <col min="16" max="16" width="9.109375" customWidth="1"/>
+    <col min="17" max="17" width="14.88671875" customWidth="1"/>
+    <col min="18" max="18" width="18.5546875" customWidth="1"/>
+    <col min="19" max="19" width="18.88671875" customWidth="1"/>
+    <col min="20" max="20" width="18.33203125" customWidth="1"/>
+    <col min="21" max="21" width="23.6640625" customWidth="1"/>
+    <col min="22" max="22" width="18.88671875" customWidth="1"/>
+    <col min="23" max="23" width="17.77734375" customWidth="1"/>
+    <col min="24" max="24" width="15.33203125" customWidth="1"/>
+    <col min="25" max="25" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B2">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="1">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" t="s">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <v>0</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
       </c>
       <c r="N2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="Q2" t="s">
-        <v>24</v>
-      </c>
-      <c r="R2">
+        <v>25</v>
+      </c>
+      <c r="R2" s="2">
         <v>0</v>
       </c>
       <c r="S2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="U2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="V2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="W2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="X2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>